<commit_message>
Delegate edition: council rework (safety guardrails, four-tier classification, cut to 2.2k words, humor pass); sample Excel with FAKE- IDs and watermark
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/portfolio_sample.xlsx
+++ b/portfolio_sample.xlsx
@@ -31,14 +31,16 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00991B1B"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00991B1B"/>
       <sz val="13"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -68,9 +70,9 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -437,72 +439,67 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Sample portfolio data for the AI Tuesday edition 'Delegate, don't chat'.</t>
+          <t>INVENTED DATA FOR TESTING ONLY (AI Tuesday, 'Delegate, don't chat')</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Everything here is invented: project IDs, names, TTLs, amounts. Use it to try the Analyst agent in Microsoft 365 Copilot.</t>
+          <t>Every project, ID (FAKE-1001 to FAKE-1024), amount, date and name in this file is fictional. The TTLs are dead scientists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Use it to try the Analyst agent in Microsoft 365 Copilot. Then delete it, and start a NEW chat before attaching a real file.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Try asking Analyst:</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1. Which projects are behind on disbursement relative to time elapsed? Rank them and explain the method.</t>
+          <t>Sheets: Portfolio (24 projects) and Disbursement history (semi-annual, up to 2026-H1).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2. Total commitments and disbursement rate by sector and by country, with a chart.</t>
-        </is>
-      </c>
+      <c r="A7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>3. Which projects close in the next 12 months with less than 70% disbursed?</t>
+          <t>The one brief to paste into Analyst (attach this file first):</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>4. Using the Disbursement history sheet, which projects are accelerating and which are slowing down?</t>
+          <t>Using the attached portfolio file: for each project, compute the share of time elapsed between effectiveness and revised closing date as of 6 October 2026, and the share of commitment disbursed. Rank projects by the gap (time elapsed minus disbursed), largest first. Show a table and a scatter chart with project IDs as labels. Then list the projects closing within 12 months that are below 70% disbursed (70% is an illustration, not a Bank threshold). First tell me how many projects you included and which columns you used. Explain your method in three sentences.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>5. Write a one-paragraph portfolio summary for a Country Director.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Check one answer by hand before you trust the rest. That is the whole point.</t>
+      <c r="A10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Then check two things by hand: one project's disbursement rate, and the project count (24).</t>
         </is>
       </c>
     </row>
@@ -517,281 +514,244 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>INVENTED DATA FOR TESTING ONLY. Every project, ID, amount and name on this sheet is fictional. Delete after testing. Start a new chat before attaching your real file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Project ID</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Sector</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Project name</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Commitment (USD M)</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Disbursed (USD M)</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Effectiveness date</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
-        <is>
-          <t>Closing date</t>
-        </is>
-      </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Revised closing date</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>Risk rating</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
-        <is>
-          <t>TTL</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>P179096</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Honduras</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Social Protection</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Youth Employment Project</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>150</v>
-      </c>
-      <c r="F2" t="n">
-        <v>32.2</v>
-      </c>
-      <c r="G2" s="4" t="n">
-        <v>45530</v>
-      </c>
-      <c r="H2" s="4" t="n">
-        <v>46990</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>A. Rivera</t>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>TTL (fictional)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>P173910</t>
+          <t>FAKE-1001</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>Dominican Republic</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Urban</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Early Childhood Project</t>
+          <t>Urban Resilience Project</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>20</v>
+        <v>250</v>
       </c>
       <c r="F3" t="n">
-        <v>17.6</v>
+        <v>92.3</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>44373</v>
+        <v>45399</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>46198</v>
+        <v>46859</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>A. Rivera</t>
+          <t>Alan Turing</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>P172998</t>
+          <t>FAKE-1002</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Urban</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Secondary Education Quality Project</t>
+          <t>Urban Resilience Project</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="F4" t="n">
-        <v>25.5</v>
+        <v>48.6</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>45488</v>
+        <v>44382</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>47678</v>
+        <v>46572</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Substantial</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>A. Rivera</t>
+          <t>Ada Lovelace</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>P170108</t>
+          <t>FAKE-1003</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bolivia</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Agriculture</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Secondary Education Quality Project</t>
+          <t>Irrigation Modernization Project</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="F5" t="n">
-        <v>220.1</v>
+        <v>156.7</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>44469</v>
+        <v>45528</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>46294</v>
+        <v>46988</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Substantial</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>L. Okafor</t>
+          <t>Rosalind Franklin</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>P166748</t>
+          <t>FAKE-1004</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Peru</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Secondary Education Quality Project</t>
+          <t>Rural Learning Project</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>120</v>
+        <v>75</v>
       </c>
       <c r="F6" t="n">
-        <v>109.1</v>
+        <v>50.8</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>44396</v>
+        <v>45425</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>46586</v>
+        <v>46885</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -800,42 +760,42 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>E. Moreau</t>
+          <t>Grace Hopper</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>P165890</t>
+          <t>FAKE-1005</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Agriculture</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Clean Energy Access Project</t>
+          <t>Rural Sanitation Project</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>120</v>
+        <v>200</v>
       </c>
       <c r="F7" t="n">
-        <v>81.7</v>
+        <v>130.7</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>45150</v>
+        <v>44206</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>47340</v>
+        <v>46396</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -844,130 +804,130 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>S. Haddad</t>
+          <t>Hypatia of Alexandria</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>P163868</t>
+          <t>FAKE-1006</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Transport</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Primary Health Strengthening Project</t>
+          <t>Maternal and Child Health Project</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>250</v>
+        <v>120</v>
       </c>
       <c r="F8" t="n">
-        <v>161.6</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>45210</v>
+        <v>44667</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>47035</v>
+        <v>46857</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>C. Duarte</t>
+          <t>Rosalind Franklin</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>P178776</t>
+          <t>FAKE-1007</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Early Childhood Project</t>
+          <t>Maternal and Child Health Project</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="F9" t="n">
-        <v>13.7</v>
+        <v>150</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>45198</v>
+        <v>44333</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>47023</v>
+        <v>45793</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Substantial</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>P. Singh</t>
+          <t>Grace Hopper</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>P168845</t>
+          <t>FAKE-1008</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Honduras</t>
+          <t>Peru</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Urban</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Primary Health Strengthening Project</t>
+          <t>Urban Resilience Project</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>300</v>
+        <v>150</v>
       </c>
       <c r="F10" t="n">
-        <v>174.7</v>
+        <v>122.1</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>45214</v>
+        <v>45056</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>47404</v>
+        <v>46516</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -976,19 +936,19 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>E. Moreau</t>
+          <t>Marie Curie</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>P169325</t>
+          <t>FAKE-1009</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>El Salvador</t>
+          <t>Honduras</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -998,85 +958,85 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Digital Government Project</t>
+          <t>Maternal and Child Health Project</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>20</v>
+        <v>120</v>
       </c>
       <c r="F11" t="n">
-        <v>12.7</v>
+        <v>120</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>44831</v>
+        <v>44228</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>47021</v>
+        <v>46053</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Substantial</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>C. Duarte</t>
+          <t>Grace Hopper</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>P167150</t>
+          <t>FAKE-1010</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>El Salvador</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Rural Learning Project</t>
+          <t>Primary Health Strengthening Project</t>
         </is>
       </c>
       <c r="E12" t="n">
         <v>20</v>
       </c>
       <c r="F12" t="n">
-        <v>7.5</v>
+        <v>7.6</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>45142</v>
+        <v>45149</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>46967</v>
+        <v>46974</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>J. Novak</t>
+          <t>Nikola Tesla</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>P169104</t>
+          <t>FAKE-1011</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1086,20 +1046,20 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Early Childhood Project</t>
+          <t>Urban Water Supply Project</t>
         </is>
       </c>
       <c r="E13" t="n">
         <v>150</v>
       </c>
       <c r="F13" t="n">
-        <v>60.9</v>
+        <v>21.7</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>44997</v>
+        <v>45515</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>46822</v>
+        <v>47340</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -1108,19 +1068,19 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>L. Okafor</t>
+          <t>Grace Hopper</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>P162719</t>
+          <t>FAKE-1012</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Guatemala</t>
+          <t>Peru</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1130,80 +1090,80 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Resilient Roads Project</t>
+          <t>Rural Access Roads Project</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>150</v>
+        <v>20</v>
       </c>
       <c r="F14" t="n">
-        <v>113.9</v>
+        <v>17.3</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>44931</v>
+        <v>44628</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>47121</v>
+        <v>46088</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Substantial</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>L. Okafor</t>
+          <t>Rosalind Franklin</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>P160134</t>
+          <t>FAKE-1013</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Peru</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Social Protection</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Urban Water Supply Project</t>
+          <t>Youth Employment Project</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>75</v>
+        <v>200</v>
       </c>
       <c r="F15" t="n">
-        <v>75</v>
+        <v>200</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>44221</v>
+        <v>44725</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>46046</v>
+        <v>46185</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>L. Okafor</t>
+          <t>Marie Curie</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>P161769</t>
+          <t>FAKE-1014</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1213,69 +1173,69 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Early Childhood Project</t>
+          <t>Primary Health Strengthening Project</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>300</v>
+        <v>35</v>
       </c>
       <c r="F16" t="n">
-        <v>206.8</v>
+        <v>26.8</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>45356</v>
+        <v>44624</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>47181</v>
+        <v>46814</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Substantial</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>E. Moreau</t>
+          <t>Isaac Newton</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>P166245</t>
+          <t>FAKE-1015</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Honduras</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Agriculture</t>
+          <t>Urban</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Rural Learning Project</t>
+          <t>Secondary Cities Development Project</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="F17" t="n">
-        <v>61.4</v>
+        <v>70</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>45014</v>
+        <v>45187</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>46839</v>
+        <v>47377</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1284,190 +1244,190 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>M. Chen</t>
+          <t>Alan Turing</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>P164956</t>
+          <t>FAKE-1016</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Bolivia</t>
+          <t>Paraguay</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Secondary Education Quality Project</t>
+          <t>Urban Water Supply Project</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="F18" t="n">
-        <v>49</v>
+        <v>60.7</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>44422</v>
+        <v>44521</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>46247</v>
+        <v>46711</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>M. Chen</t>
+          <t>Hypatia of Alexandria</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>P179735</t>
+          <t>FAKE-1017</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Honduras</t>
+          <t>Dominican Republic</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Youth Employment Project</t>
+          <t>Maternal and Child Health Project</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="F19" t="n">
-        <v>21.7</v>
+        <v>13.4</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>44622</v>
+        <v>44409</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>46812</v>
+        <v>45869</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>P. Singh</t>
+          <t>Grace Hopper</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>P163348</t>
+          <t>FAKE-1018</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>El Salvador</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Agriculture</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Resilient Roads Project</t>
+          <t>Irrigation Modernization Project</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>35</v>
+        <v>150</v>
       </c>
       <c r="F20" t="n">
-        <v>18.1</v>
+        <v>44.3</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>45196</v>
+        <v>45418</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>47021</v>
+        <v>47243</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>P. Singh</t>
+          <t>Rosalind Franklin</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>P171853</t>
+          <t>FAKE-1019</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>El Salvador</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Transport</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Early Childhood Project</t>
+          <t>Rural Sanitation Project</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="F21" t="n">
-        <v>94.09999999999999</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>44527</v>
+        <v>45535</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>46717</v>
+        <v>47725</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>L. Okafor</t>
+          <t>Grace Hopper</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>P176986</t>
+          <t>FAKE-1020</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1482,64 +1442,64 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Urban Water Supply Project</t>
+          <t>Rural Learning Project</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>250</v>
+        <v>100</v>
       </c>
       <c r="F22" t="n">
-        <v>201.2</v>
+        <v>47.8</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>44807</v>
+        <v>45039</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>46997</v>
+        <v>46864</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Substantial</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>P. Singh</t>
+          <t>Marie Curie</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>P166394</t>
+          <t>FAKE-1021</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Honduras</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Social Protection</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Clean Energy Access Project</t>
+          <t>Youth Employment Project</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>75</v>
+        <v>120</v>
       </c>
       <c r="F23" t="n">
-        <v>40.4</v>
+        <v>120</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>45287</v>
+        <v>44480</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>47477</v>
+        <v>46305</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -1548,24 +1508,24 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>S. Haddad</t>
+          <t>Alan Turing</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>P169155</t>
+          <t>FAKE-1022</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Guatemala</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1574,16 +1534,16 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>75</v>
+        <v>200</v>
       </c>
       <c r="F24" t="n">
-        <v>31.1</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>45257</v>
+        <v>44929</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>47082</v>
+        <v>47119</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -1592,51 +1552,95 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>E. Moreau</t>
+          <t>Rosalind Franklin</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>P171948</t>
+          <t>FAKE-1023</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Paraguay</t>
+          <t>El Salvador</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Youth Employment Project</t>
+          <t>Early Childhood Development Project</t>
         </is>
       </c>
       <c r="E25" t="n">
+        <v>50</v>
+      </c>
+      <c r="F25" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>44896</v>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>46721</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Rosalind Franklin</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>FAKE-1024</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Guatemala</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Secondary Education Quality Project</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
         <v>300</v>
       </c>
-      <c r="F25" t="n">
-        <v>257.6</v>
-      </c>
-      <c r="G25" s="4" t="n">
-        <v>44902</v>
-      </c>
-      <c r="H25" s="4" t="n">
-        <v>46727</v>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>Substantial</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>M. Chen</t>
+      <c r="F26" t="n">
+        <v>288.5</v>
+      </c>
+      <c r="G26" s="4" t="n">
+        <v>44226</v>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>46416</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Ada Lovelace</t>
         </is>
       </c>
     </row>
@@ -1651,110 +1655,102 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C171"/>
+  <dimension ref="A1:C180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>INVENTED DATA FOR TESTING ONLY. Every project, ID, amount and name on this sheet is fictional. Delete after testing. Start a new chat before attaching your real file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Project ID</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Disbursed in period (USD M)</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>P179096</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2025-H1</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>P179096</t>
+          <t>FAKE-1001</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2025-H2</t>
+          <t>2024-H2</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>8.300000000000001</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>P179096</t>
+          <t>FAKE-1001</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-H1</t>
+          <t>2025-H1</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7.7</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>P179096</t>
+          <t>FAKE-1001</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-H2</t>
+          <t>2025-H2</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>7.9</v>
+        <v>24.8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>P173910</t>
+          <t>FAKE-1001</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2021-H2</t>
+          <t>2026-H1</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.7</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>P173910</t>
+          <t>FAKE-1002</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1763,13 +1759,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2.2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>P173910</t>
+          <t>FAKE-1002</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1778,13 +1774,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2.1</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>P173910</t>
+          <t>FAKE-1002</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1793,13 +1789,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1.4</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>P173910</t>
+          <t>FAKE-1002</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1808,13 +1804,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1.7</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>P173910</t>
+          <t>FAKE-1002</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1823,13 +1819,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>P173910</t>
+          <t>FAKE-1002</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1838,1063 +1834,1063 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>P173910</t>
+          <t>FAKE-1002</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2025-H1</t>
+          <t>2024-H2</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1.7</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>P173910</t>
+          <t>FAKE-1002</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2025-H2</t>
+          <t>2025-H1</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2.2</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>P173910</t>
+          <t>FAKE-1002</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-H1</t>
+          <t>2025-H2</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>P172998</t>
+          <t>FAKE-1002</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2025-H1</t>
+          <t>2026-H1</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>8.1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>P172998</t>
+          <t>FAKE-1003</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2025-H2</t>
+          <t>2025-H1</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>5.8</v>
+        <v>44.7</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>P172998</t>
+          <t>FAKE-1003</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-H1</t>
+          <t>2025-H2</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>3.2</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>P172998</t>
+          <t>FAKE-1003</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-H2</t>
+          <t>2026-H1</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>8.4</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>P170108</t>
+          <t>FAKE-1003</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2022-H1</t>
+          <t>2026-H2</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>16.7</v>
+        <v>50.1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>P170108</t>
+          <t>FAKE-1004</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2022-H2</t>
+          <t>2024-H2</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>31.4</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>P170108</t>
+          <t>FAKE-1004</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2023-H1</t>
+          <t>2025-H1</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>36.7</v>
+        <v>13.4</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>P170108</t>
+          <t>FAKE-1004</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2023-H2</t>
+          <t>2025-H2</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>18.7</v>
+        <v>18.4</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>P170108</t>
+          <t>FAKE-1004</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2024-H1</t>
+          <t>2026-H1</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>18.9</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>P170108</t>
+          <t>FAKE-1005</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2024-H2</t>
+          <t>2021-H2</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>35.9</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>P170108</t>
+          <t>FAKE-1005</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2025-H1</t>
+          <t>2022-H1</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>29</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>P170108</t>
+          <t>FAKE-1005</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2025-H2</t>
+          <t>2022-H2</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>11.6</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>P170108</t>
+          <t>FAKE-1005</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-H1</t>
+          <t>2023-H1</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>10.3</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>P170108</t>
+          <t>FAKE-1005</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-H2</t>
+          <t>2023-H2</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>11</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>P166748</t>
+          <t>FAKE-1005</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2022-H1</t>
+          <t>2024-H1</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>16.4</v>
+        <v>19.4</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>P166748</t>
+          <t>FAKE-1005</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2022-H2</t>
+          <t>2024-H2</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>14.9</v>
+        <v>15.1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>P166748</t>
+          <t>FAKE-1005</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2023-H1</t>
+          <t>2025-H1</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>5.1</v>
+        <v>11.3</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>P166748</t>
+          <t>FAKE-1005</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2023-H2</t>
+          <t>2025-H2</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>15.2</v>
+        <v>19.1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>P166748</t>
+          <t>FAKE-1005</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2024-H1</t>
+          <t>2026-H1</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>17.5</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>P166748</t>
+          <t>FAKE-1005</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2024-H2</t>
+          <t>2026-H2</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>12.7</v>
+        <v>15.2</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>P166748</t>
+          <t>FAKE-1006</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2025-H1</t>
+          <t>2022-H2</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>8.199999999999999</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>P166748</t>
+          <t>FAKE-1006</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2025-H2</t>
+          <t>2023-H1</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>11.1</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>P166748</t>
+          <t>FAKE-1006</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-H1</t>
+          <t>2023-H2</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>4.9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>P166748</t>
+          <t>FAKE-1006</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-H2</t>
+          <t>2024-H1</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3.2</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>P165890</t>
+          <t>FAKE-1006</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2024-H1</t>
+          <t>2024-H2</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>17.1</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>P165890</t>
+          <t>FAKE-1006</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2024-H2</t>
+          <t>2025-H1</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>12.4</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>P165890</t>
+          <t>FAKE-1006</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2025-H1</t>
+          <t>2025-H2</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>10.6</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>P165890</t>
+          <t>FAKE-1006</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2025-H2</t>
+          <t>2026-H1</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>16.6</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>P165890</t>
+          <t>FAKE-1007</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-H1</t>
+          <t>2021-H2</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>9.300000000000001</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>P165890</t>
+          <t>FAKE-1007</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-H2</t>
+          <t>2022-H1</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>15.7</v>
+        <v>14.6</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>P163868</t>
+          <t>FAKE-1007</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2024-H1</t>
+          <t>2022-H2</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>58.8</v>
+        <v>21.8</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>P163868</t>
+          <t>FAKE-1007</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2024-H2</t>
+          <t>2023-H1</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>23.5</v>
+        <v>22</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>P163868</t>
+          <t>FAKE-1007</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2025-H1</t>
+          <t>2023-H2</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>25.9</v>
+        <v>19.1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>P163868</t>
+          <t>FAKE-1007</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2025-H2</t>
+          <t>2024-H1</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>28.2</v>
+        <v>24.1</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>P163868</t>
+          <t>FAKE-1007</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-H1</t>
+          <t>2024-H2</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>25.2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>P178776</t>
+          <t>FAKE-1007</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2024-H1</t>
+          <t>2025-H1</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2.8</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>P178776</t>
+          <t>FAKE-1007</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2024-H2</t>
+          <t>2025-H2</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1.6</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>P178776</t>
+          <t>FAKE-1007</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2025-H1</t>
+          <t>2026-H1</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>2.2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>P178776</t>
+          <t>FAKE-1008</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2025-H2</t>
+          <t>2023-H2</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1.2</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>P178776</t>
+          <t>FAKE-1008</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-H1</t>
+          <t>2024-H1</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>3.9</v>
+        <v>18.3</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>P178776</t>
+          <t>FAKE-1008</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-H2</t>
+          <t>2024-H2</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>2</v>
+        <v>24.6</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>P168845</t>
+          <t>FAKE-1008</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2024-H1</t>
+          <t>2025-H1</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>26.8</v>
+        <v>20.7</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>P168845</t>
+          <t>FAKE-1008</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2024-H2</t>
+          <t>2025-H2</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>31.9</v>
+        <v>15.3</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>P168845</t>
+          <t>FAKE-1008</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2025-H1</t>
+          <t>2026-H1</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>45</v>
+        <v>30.9</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>P168845</t>
+          <t>FAKE-1009</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2025-H2</t>
+          <t>2021-H2</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>25.3</v>
+        <v>20.1</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>P168845</t>
+          <t>FAKE-1009</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-H1</t>
+          <t>2022-H1</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>45.6</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>P169325</t>
+          <t>FAKE-1009</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2023-H1</t>
+          <t>2022-H2</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1.9</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>P169325</t>
+          <t>FAKE-1009</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2023-H2</t>
+          <t>2023-H1</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>2</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>P169325</t>
+          <t>FAKE-1009</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2024-H1</t>
+          <t>2023-H2</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>2</v>
+        <v>18.3</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>P169325</t>
+          <t>FAKE-1009</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2024-H2</t>
+          <t>2024-H1</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>0.6</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>P169325</t>
+          <t>FAKE-1009</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2025-H1</t>
+          <t>2024-H2</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1.8</v>
+        <v>15.5</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>P169325</t>
+          <t>FAKE-1009</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2025-H2</t>
+          <t>2025-H1</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1.1</v>
+        <v>13.1</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>P169325</t>
+          <t>FAKE-1009</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-H1</t>
+          <t>2025-H2</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>0.6</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>P169325</t>
+          <t>FAKE-1009</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-H2</t>
+          <t>2026-H1</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>2.8</v>
+        <v>16.9</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>P167150</t>
+          <t>FAKE-1009</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2024-H1</t>
+          <t>2026-H2</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>0.7</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>P167150</t>
+          <t>FAKE-1010</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2024-H2</t>
+          <t>2024-H1</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>1.3</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>P167150</t>
+          <t>FAKE-1010</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2025-H1</t>
+          <t>2024-H2</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>P167150</t>
+          <t>FAKE-1010</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2025-H2</t>
+          <t>2025-H1</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>1.4</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>P167150</t>
+          <t>FAKE-1010</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-H1</t>
+          <t>2025-H2</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>1</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>P167150</t>
+          <t>FAKE-1010</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-H2</t>
+          <t>2026-H1</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1.4</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>P169104</t>
+          <t>FAKE-1010</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2023-H2</t>
+          <t>2026-H2</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>9.800000000000001</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>P169104</t>
+          <t>FAKE-1011</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2024-H1</t>
+          <t>2025-H1</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>12.7</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>P169104</t>
+          <t>FAKE-1011</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2024-H2</t>
+          <t>2025-H2</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>P169104</t>
+          <t>FAKE-1011</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2025-H1</t>
+          <t>2026-H1</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>9.800000000000001</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>P169104</t>
+          <t>FAKE-1011</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2025-H2</t>
+          <t>2026-H2</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>5.8</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>P169104</t>
+          <t>FAKE-1012</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-H1</t>
+          <t>2022-H2</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>6.2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>P169104</t>
+          <t>FAKE-1012</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-H2</t>
+          <t>2023-H1</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>12.6</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>P162719</t>
+          <t>FAKE-1012</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2903,13 +2899,13 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>14.1</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>P162719</t>
+          <t>FAKE-1012</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2918,13 +2914,13 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>15.2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>P162719</t>
+          <t>FAKE-1012</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2933,13 +2929,13 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>19.2</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>P162719</t>
+          <t>FAKE-1012</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2948,13 +2944,13 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>22.2</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>P162719</t>
+          <t>FAKE-1012</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2963,13 +2959,13 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>12.8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>P162719</t>
+          <t>FAKE-1012</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2978,13 +2974,13 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>16.2</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>P162719</t>
+          <t>FAKE-1012</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2993,268 +2989,268 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>14.1</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>P160134</t>
+          <t>FAKE-1013</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2021-H2</t>
+          <t>2022-H2</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>5.8</v>
+        <v>32.1</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>P160134</t>
+          <t>FAKE-1013</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2022-H1</t>
+          <t>2023-H1</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>7.3</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>P160134</t>
+          <t>FAKE-1013</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2022-H2</t>
+          <t>2023-H2</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>5.3</v>
+        <v>16.6</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>P160134</t>
+          <t>FAKE-1013</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2023-H1</t>
+          <t>2024-H1</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>6</v>
+        <v>19.1</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>P160134</t>
+          <t>FAKE-1013</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2023-H2</t>
+          <t>2024-H2</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>5.6</v>
+        <v>31.5</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>P160134</t>
+          <t>FAKE-1013</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2024-H1</t>
+          <t>2025-H1</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>9.4</v>
+        <v>25.3</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>P160134</t>
+          <t>FAKE-1013</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2024-H2</t>
+          <t>2025-H2</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>7.4</v>
+        <v>28.6</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>P160134</t>
+          <t>FAKE-1013</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2025-H1</t>
+          <t>2026-H1</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>8.800000000000001</v>
+        <v>33.6</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>P160134</t>
+          <t>FAKE-1014</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2025-H2</t>
+          <t>2022-H2</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>9.4</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>P160134</t>
+          <t>FAKE-1014</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-H1</t>
+          <t>2023-H1</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>3.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>P160134</t>
+          <t>FAKE-1014</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-H2</t>
+          <t>2023-H2</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>6.2</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>P161769</t>
+          <t>FAKE-1014</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2024-H2</t>
+          <t>2024-H1</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>67.90000000000001</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>P161769</t>
+          <t>FAKE-1014</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2025-H1</t>
+          <t>2024-H2</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>61.7</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>P161769</t>
+          <t>FAKE-1014</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2025-H2</t>
+          <t>2025-H1</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>20</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>P161769</t>
+          <t>FAKE-1014</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-H1</t>
+          <t>2025-H2</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>19.1</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>P161769</t>
+          <t>FAKE-1014</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-H2</t>
+          <t>2026-H1</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>38.1</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>P166245</t>
+          <t>FAKE-1014</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2023-H2</t>
+          <t>2026-H2</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>3.9</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>P166245</t>
+          <t>FAKE-1015</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3263,13 +3259,13 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>6.3</v>
+        <v>13.7</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>P166245</t>
+          <t>FAKE-1015</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3278,13 +3274,13 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>3.9</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>P166245</t>
+          <t>FAKE-1015</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3293,13 +3289,13 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>12.4</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>P166245</t>
+          <t>FAKE-1015</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3308,13 +3304,13 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>14.1</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>P166245</t>
+          <t>FAKE-1015</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3323,13 +3319,13 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>15.7</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>P166245</t>
+          <t>FAKE-1015</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3338,13 +3334,13 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>5.1</v>
+        <v>14.1</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>P164956</t>
+          <t>FAKE-1016</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -3353,13 +3349,13 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>5.3</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>P164956</t>
+          <t>FAKE-1016</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3368,13 +3364,13 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>5</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>P164956</t>
+          <t>FAKE-1016</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3383,13 +3379,13 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>2</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>P164956</t>
+          <t>FAKE-1016</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3398,13 +3394,13 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>6.3</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>P164956</t>
+          <t>FAKE-1016</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3413,13 +3409,13 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>6.8</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>P164956</t>
+          <t>FAKE-1016</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3428,13 +3424,13 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>2.4</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>P164956</t>
+          <t>FAKE-1016</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -3443,13 +3439,13 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>6.7</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>P164956</t>
+          <t>FAKE-1016</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3464,7 +3460,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>P164956</t>
+          <t>FAKE-1016</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3473,28 +3469,28 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>4</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>P164956</t>
+          <t>FAKE-1017</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-H2</t>
+          <t>2022-H1</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>6.9</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>P179735</t>
+          <t>FAKE-1017</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3503,13 +3499,13 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>4.2</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>P179735</t>
+          <t>FAKE-1017</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3518,13 +3514,13 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>P179735</t>
+          <t>FAKE-1017</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3533,13 +3529,13 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>2.6</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>P179735</t>
+          <t>FAKE-1017</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3548,13 +3544,13 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>2.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>P179735</t>
+          <t>FAKE-1017</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3563,13 +3559,13 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>2.2</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>P179735</t>
+          <t>FAKE-1017</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3578,13 +3574,13 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>P179735</t>
+          <t>FAKE-1017</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3593,13 +3589,13 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>2.1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>P179735</t>
+          <t>FAKE-1017</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3608,13 +3604,13 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>3.8</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>P179735</t>
+          <t>FAKE-1017</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3623,607 +3619,742 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>P163348</t>
+          <t>FAKE-1018</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2024-H1</t>
+          <t>2024-H2</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>3.7</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>P163348</t>
+          <t>FAKE-1018</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2024-H2</t>
+          <t>2025-H1</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>3.1</v>
+        <v>16.3</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>P163348</t>
+          <t>FAKE-1018</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2025-H1</t>
+          <t>2025-H2</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>1.1</v>
+        <v>11.6</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>P163348</t>
+          <t>FAKE-1018</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2025-H2</t>
+          <t>2026-H1</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>2.6</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>P163348</t>
+          <t>FAKE-1019</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-H1</t>
+          <t>2025-H1</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>4.1</v>
+        <v>32.2</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>P163348</t>
+          <t>FAKE-1019</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-H2</t>
+          <t>2025-H2</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>3.5</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>P171853</t>
+          <t>FAKE-1019</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2022-H1</t>
+          <t>2026-H1</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>4.1</v>
+        <v>31.9</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>P171853</t>
+          <t>FAKE-1019</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2022-H2</t>
+          <t>2026-H2</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>18.4</v>
+        <v>11.9</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>P171853</t>
+          <t>FAKE-1020</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2023-H1</t>
+          <t>2023-H2</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>15.3</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>P171853</t>
+          <t>FAKE-1020</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2023-H2</t>
+          <t>2024-H1</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>18.2</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>P171853</t>
+          <t>FAKE-1020</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2024-H1</t>
+          <t>2024-H2</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>4.7</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>P171853</t>
+          <t>FAKE-1020</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2024-H2</t>
+          <t>2025-H1</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>7.2</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>P171853</t>
+          <t>FAKE-1020</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2025-H1</t>
+          <t>2025-H2</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>3.7</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>P171853</t>
+          <t>FAKE-1020</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2025-H2</t>
+          <t>2026-H1</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>15.2</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>P171853</t>
+          <t>FAKE-1021</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-H1</t>
+          <t>2022-H1</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>7.3</v>
+        <v>16.1</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>P176986</t>
+          <t>FAKE-1021</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2023-H1</t>
+          <t>2022-H2</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>11.5</v>
+        <v>13.7</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>P176986</t>
+          <t>FAKE-1021</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2023-H2</t>
+          <t>2023-H1</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>21.7</v>
+        <v>17.7</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>P176986</t>
+          <t>FAKE-1021</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2024-H1</t>
+          <t>2023-H2</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>38.7</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>P176986</t>
+          <t>FAKE-1021</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2024-H2</t>
+          <t>2024-H1</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>35.5</v>
+        <v>17.7</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>P176986</t>
+          <t>FAKE-1021</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2025-H1</t>
+          <t>2024-H2</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>16</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>P176986</t>
+          <t>FAKE-1021</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2025-H2</t>
+          <t>2025-H1</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>12.2</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>P176986</t>
+          <t>FAKE-1021</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-H1</t>
+          <t>2025-H2</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>39</v>
+        <v>11.2</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>P176986</t>
+          <t>FAKE-1021</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-H2</t>
+          <t>2026-H1</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>26.8</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>P166394</t>
+          <t>FAKE-1021</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2024-H1</t>
+          <t>2026-H2</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>12.3</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>P166394</t>
+          <t>FAKE-1022</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2024-H2</t>
+          <t>2023-H2</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>3.9</v>
+        <v>13.7</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>P166394</t>
+          <t>FAKE-1022</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2025-H1</t>
+          <t>2024-H1</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>3.5</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>P166394</t>
+          <t>FAKE-1022</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2025-H2</t>
+          <t>2024-H2</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>12.1</v>
+        <v>17</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>P166394</t>
+          <t>FAKE-1022</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-H1</t>
+          <t>2024-H2</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>8.5</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>P169155</t>
+          <t>FAKE-1022</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2024-H1</t>
+          <t>2025-H2</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>2.4</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>P169155</t>
+          <t>FAKE-1022</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2024-H2</t>
+          <t>2025-H2</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>10</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>P169155</t>
+          <t>FAKE-1022</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2025-H1</t>
+          <t>2026-H1</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>7.4</v>
+        <v>17</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>P169155</t>
+          <t>FAKE-1023</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2025-H2</t>
+          <t>2023-H1</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>8.800000000000001</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>P169155</t>
+          <t>FAKE-1023</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-H1</t>
+          <t>2023-H2</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>2.5</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>P171948</t>
+          <t>FAKE-1023</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2023-H1</t>
+          <t>2024-H1</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>49.8</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>P171948</t>
+          <t>FAKE-1023</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2023-H2</t>
+          <t>2024-H2</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>12.6</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>P171948</t>
+          <t>FAKE-1023</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2024-H1</t>
+          <t>2025-H1</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>50.2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>P171948</t>
+          <t>FAKE-1023</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2024-H2</t>
+          <t>2025-H2</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>30.9</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>P171948</t>
+          <t>FAKE-1023</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2025-H1</t>
+          <t>2026-H1</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>25.4</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>P171948</t>
+          <t>FAKE-1024</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2025-H2</t>
+          <t>2021-H2</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>35.5</v>
+        <v>25.6</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>P171948</t>
+          <t>FAKE-1024</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
+          <t>2022-H1</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>24.4</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>FAKE-1024</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>2022-H2</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>FAKE-1024</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>2023-H1</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>FAKE-1024</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>2023-H2</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>40.6</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>FAKE-1024</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>2024-H1</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>24.9</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>FAKE-1024</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>2024-H2</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>20.9</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>FAKE-1024</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>2025-H1</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>34.8</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>FAKE-1024</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>2025-H2</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>26.5</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>FAKE-1024</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
           <t>2026-H1</t>
         </is>
       </c>
-      <c r="C171" t="n">
-        <v>53.2</v>
+      <c r="C179" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>FAKE-1024</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>2026-H2</t>
+        </is>
+      </c>
+      <c r="C180" t="n">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>